<commit_message>
about to overhaul placeholder logic
</commit_message>
<xml_diff>
--- a/AhMen Client Data and Docs Template.xlsx
+++ b/AhMen Client Data and Docs Template.xlsx
@@ -5,12 +5,12 @@
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/motticohen/Dropbox/AhMen Admin/*CLIENT DATA/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/motticohen/Desktop/invoice_master_dashboard/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D706930A-F618-AA42-B3FA-A50882B9590C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A32A114-CE6B-154D-B8DF-A654DAC6E6D6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="23000" yWindow="500" windowWidth="27160" windowHeight="28300" activeTab="6" xr2:uid="{B5763DD8-C14C-9E43-BCE3-8FC2FCC62202}"/>
+    <workbookView xWindow="23000" yWindow="500" windowWidth="27160" windowHeight="28300" activeTab="3" xr2:uid="{B5763DD8-C14C-9E43-BCE3-8FC2FCC62202}"/>
   </bookViews>
   <sheets>
     <sheet name="Client Data" sheetId="3" r:id="rId1"/>
@@ -5183,7 +5183,7 @@
       <c r="D6" s="26"/>
       <c r="E6" s="27">
         <f ca="1">TODAY()</f>
-        <v>45919</v>
+        <v>45921</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -7445,7 +7445,7 @@
       <c r="D6" s="26"/>
       <c r="E6" s="27">
         <f ca="1">TODAY()</f>
-        <v>45919</v>
+        <v>45921</v>
       </c>
     </row>
     <row r="7" spans="2:8" ht="15" customHeight="1" x14ac:dyDescent="0.2">
@@ -7694,7 +7694,7 @@
       </c>
       <c r="C33" s="15">
         <f ca="1">TODAY()</f>
-        <v>45919</v>
+        <v>45921</v>
       </c>
       <c r="I33" s="6"/>
     </row>

</xml_diff>